<commit_message>
Commit of newwest reporting format and email changes
</commit_message>
<xml_diff>
--- a/resources/reports/weekly-report-template.xlsx
+++ b/resources/reports/weekly-report-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly report" sheetId="1" r:id="R397acc6b39e34eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly report" sheetId="1" r:id="R389c7f069fa743ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -149,8 +149,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BarristerRequests" displayName="BarristerRequests" ref="A6:G7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A6:G7"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BarristerRequests" displayName="BarristerRequests" ref="A1:G2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G2"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Barrister name"/>
     <x:tableColumn id="2" name="Email address"/>
@@ -371,96 +371,87 @@
     <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2"/>
-      <x:c r="B1" s="2"/>
-      <x:c r="C1" s="2"/>
-      <x:c r="D1" s="2"/>
-      <x:c r="E1" s="2"/>
-      <x:c r="F1" s="2"/>
-      <x:c r="G1" s="2"/>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="4" t="str">
-        <x:v>Foley's List dry cleaning report</x:v>
-      </x:c>
-      <x:c r="B2" s="5"/>
-      <x:c r="C2" s="5"/>
-      <x:c r="D2" s="5"/>
-      <x:c r="E2" s="5"/>
-      <x:c r="F2" s="5"/>
-      <x:c r="G2" s="5"/>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Barrister name</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>Email address</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>Submitted (Melbourne)</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>Item type</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>Quantity</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>Cost (AUD)</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>Discounted cost (AUD)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="2"/>
+      <x:c r="B2" s="2"/>
+      <x:c r="C2" s="16"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="17"/>
+      <x:c r="F2" s="18"/>
+      <x:c r="G2" s="18"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="6" t="str">
-        <x:v>Requests submitted after the previous day at 5:00 pm (Australia/Melbourne).</x:v>
-      </x:c>
-      <x:c r="B3" s="2"/>
-      <x:c r="C3" s="2"/>
-      <x:c r="D3" s="2"/>
-      <x:c r="E3" s="2"/>
-      <x:c r="F3" s="2"/>
-      <x:c r="G3" s="2"/>
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+      <x:c r="F3"/>
+      <x:c r="G3"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="8" t="str">
-        <x:v>Total billed (AUD)</x:v>
-      </x:c>
-      <x:c r="B4" s="2"/>
-      <x:c r="C4" s="2"/>
-      <x:c r="D4" s="2"/>
-      <x:c r="E4" s="2"/>
-      <x:c r="F4" s="2"/>
-      <x:c r="G4" s="9" t="n">
-        <x:f>SUM(G7:G7)</x:f>
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="A4"/>
+      <x:c r="B4"/>
+      <x:c r="C4"/>
+      <x:c r="D4"/>
+      <x:c r="E4"/>
+      <x:c r="F4"/>
+      <x:c r="G4"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="2"/>
-      <x:c r="B5" s="2"/>
-      <x:c r="C5" s="2"/>
-      <x:c r="D5" s="2"/>
-      <x:c r="E5" s="2"/>
-      <x:c r="F5" s="2"/>
-      <x:c r="G5" s="2"/>
+      <x:c r="A5"/>
+      <x:c r="B5"/>
+      <x:c r="C5"/>
+      <x:c r="D5"/>
+      <x:c r="E5"/>
+      <x:c r="F5"/>
+      <x:c r="G5"/>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
-      <x:c r="A6" s="13" t="str">
-        <x:v>Barrister name</x:v>
-      </x:c>
-      <x:c r="B6" s="13" t="str">
-        <x:v>Email address</x:v>
-      </x:c>
-      <x:c r="C6" s="13" t="str">
-        <x:v>Submitted (Melbourne)</x:v>
-      </x:c>
-      <x:c r="D6" s="13" t="str">
-        <x:v>Item type</x:v>
-      </x:c>
-      <x:c r="E6" s="13" t="str">
-        <x:v>Quantity</x:v>
-      </x:c>
-      <x:c r="F6" s="13" t="str">
-        <x:v>Cost (AUD)</x:v>
-      </x:c>
-      <x:c r="G6" s="13" t="str">
-        <x:v>Discounted cost (AUD)</x:v>
-      </x:c>
+      <x:c r="A6"/>
+      <x:c r="B6"/>
+      <x:c r="C6"/>
+      <x:c r="D6"/>
+      <x:c r="E6"/>
+      <x:c r="F6"/>
+      <x:c r="G6"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="2" t="str"/>
-      <x:c r="B7" s="2" t="str"/>
-      <x:c r="C7" s="16"/>
-      <x:c r="D7" s="2" t="str"/>
-      <x:c r="E7" s="17"/>
-      <x:c r="F7" s="18"/>
-      <x:c r="G7" s="18"/>
+      <x:c r="A7"/>
+      <x:c r="B7"/>
+      <x:c r="C7"/>
+      <x:c r="D7"/>
+      <x:c r="E7"/>
+      <x:c r="F7"/>
+      <x:c r="G7"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R532bd1cad68242a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40ff091b564a43e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>